<commit_message>
chore: design patterns and DSA
</commit_message>
<xml_diff>
--- a/DSA-450-Questions/DSA 450 question Love Babbar.xlsx
+++ b/DSA-450-Questions/DSA 450 question Love Babbar.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1352" uniqueCount="465">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1352" uniqueCount="466">
   <si>
     <t>Questions by Love Babbar:</t>
   </si>
@@ -1382,6 +1382,9 @@
   </si>
   <si>
     <t>Count set bits in an integer</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>Find the two non-repeating elements in an array of repeating elements</t>
@@ -1416,13 +1419,19 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -1448,7 +1457,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -1500,43 +1509,46 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="5" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1843,9 +1855,9 @@
   <dimension ref="A1:C481"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="11" width="28.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="12" width="123.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="11" width="27.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="12" width="28.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="13" width="123.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="12" width="27.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="33">
@@ -1878,7 +1890,7 @@
         <v>4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="1"/>
       <c r="B5" s="4"/>
       <c r="C5" s="7" t="s">
@@ -6854,8 +6866,8 @@
       <c r="B472" s="9" t="s">
         <v>455</v>
       </c>
-      <c r="C472" s="7" t="s">
-        <v>5</v>
+      <c r="C472" s="11" t="s">
+        <v>456</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="473" customHeight="1" ht="18.75">
@@ -6863,7 +6875,7 @@
         <v>454</v>
       </c>
       <c r="B473" s="9" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C473" s="7" t="s">
         <v>5</v>
@@ -6874,7 +6886,7 @@
         <v>454</v>
       </c>
       <c r="B474" s="9" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="C474" s="7" t="s">
         <v>5</v>
@@ -6885,7 +6897,7 @@
         <v>454</v>
       </c>
       <c r="B475" s="9" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C475" s="7" t="s">
         <v>5</v>
@@ -6896,7 +6908,7 @@
         <v>454</v>
       </c>
       <c r="B476" s="9" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C476" s="7" t="s">
         <v>5</v>
@@ -6907,7 +6919,7 @@
         <v>454</v>
       </c>
       <c r="B477" s="9" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="C477" s="7" t="s">
         <v>5</v>
@@ -6918,7 +6930,7 @@
         <v>454</v>
       </c>
       <c r="B478" s="9" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="C478" s="7" t="s">
         <v>5</v>
@@ -6929,7 +6941,7 @@
         <v>454</v>
       </c>
       <c r="B479" s="9" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="C479" s="7" t="s">
         <v>5</v>
@@ -6940,7 +6952,7 @@
         <v>454</v>
       </c>
       <c r="B480" s="9" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C480" s="7" t="s">
         <v>5</v>
@@ -6951,7 +6963,7 @@
         <v>454</v>
       </c>
       <c r="B481" s="9" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="C481" s="7" t="s">
         <v>5</v>

</xml_diff>